<commit_message>
employee editor window. deleted the edit frame from the main window. fixed some style errors - now using a rigid style
</commit_message>
<xml_diff>
--- a/excel_files/Employees_Full_List.xlsx
+++ b/excel_files/Employees_Full_List.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="28925"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="28827"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\ScheduleApp-PyQt6\excel_files\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\bjtur\Documents\repositories\ScheduleApp-PyQt6\excel_files\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{545D3A3F-D0C4-4E74-A79B-EB37908C0541}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8BA7A6E2-D614-4CB8-A01F-C5BEB3E08777}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15990" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="525" yWindow="660" windowWidth="28800" windowHeight="15345" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="476" uniqueCount="98">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="477" uniqueCount="99">
   <si>
     <t>Name</t>
   </si>
@@ -314,6 +314,9 @@
   </si>
   <si>
     <t>Max Per Week</t>
+  </si>
+  <si>
+    <t>Time Off Dates</t>
   </si>
 </sst>
 </file>
@@ -342,7 +345,7 @@
       <patternFill patternType="gray125"/>
     </fill>
   </fills>
-  <borders count="3">
+  <borders count="2">
     <border>
       <left/>
       <right/>
@@ -365,27 +368,13 @@
       </bottom>
       <diagonal/>
     </border>
-    <border>
-      <left style="thin">
-        <color auto="1"/>
-      </left>
-      <right style="thin">
-        <color auto="1"/>
-      </right>
-      <top/>
-      <bottom/>
-      <diagonal/>
-    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="3">
+  <cellXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="top"/>
     </xf>
   </cellXfs>
@@ -690,14 +679,16 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:K86"/>
+  <dimension ref="A1:L86"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="22.5703125" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="12.42578125" bestFit="1" customWidth="1"/>
     <col min="11" max="11" width="14.140625" bestFit="1" customWidth="1"/>
+    <col min="12" max="12" width="14.28515625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -728,11 +719,14 @@
       <c r="J1" s="1" t="s">
         <v>9</v>
       </c>
-      <c r="K1" s="2" t="s">
+      <c r="K1" s="1" t="s">
         <v>97</v>
       </c>
-    </row>
-    <row r="2" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="L1" s="1" t="s">
+        <v>98</v>
+      </c>
+    </row>
+    <row r="2" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
         <v>10</v>
       </c>
@@ -764,7 +758,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="3" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
         <v>13</v>
       </c>
@@ -793,7 +787,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="4" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
         <v>14</v>
       </c>
@@ -822,7 +816,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="5" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
         <v>15</v>
       </c>
@@ -851,7 +845,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="6" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
         <v>16</v>
       </c>
@@ -874,7 +868,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="7" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
         <v>17</v>
       </c>
@@ -903,7 +897,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="8" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
         <v>18</v>
       </c>
@@ -911,7 +905,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="9" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
         <v>19</v>
       </c>
@@ -931,7 +925,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="10" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
         <v>20</v>
       </c>
@@ -951,7 +945,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="11" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A11" t="s">
         <v>21</v>
       </c>
@@ -959,7 +953,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="12" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A12" t="s">
         <v>22</v>
       </c>
@@ -979,7 +973,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="13" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A13" t="s">
         <v>23</v>
       </c>
@@ -999,7 +993,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="14" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A14" t="s">
         <v>24</v>
       </c>
@@ -1007,7 +1001,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="15" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A15" t="s">
         <v>25</v>
       </c>
@@ -1036,7 +1030,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="16" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A16" t="s">
         <v>26</v>
       </c>

</xml_diff>

<commit_message>
Fixed week not saving on draft Fixed crash and error after deleting employees
</commit_message>
<xml_diff>
--- a/excel_files/Employees_Full_List.xlsx
+++ b/excel_files/Employees_Full_List.xlsx
@@ -981,7 +981,7 @@
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>Aaron Henriksen</t>
+          <t>Colby Moon</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
@@ -989,31 +989,19 @@
           <t>Yes</t>
         </is>
       </c>
-      <c r="C15" t="inlineStr">
-        <is>
-          <t>Yes</t>
-        </is>
-      </c>
+      <c r="C15" t="inlineStr"/>
       <c r="D15" t="inlineStr">
         <is>
           <t>Yes</t>
         </is>
       </c>
-      <c r="E15" t="inlineStr">
-        <is>
-          <t>Yes</t>
-        </is>
-      </c>
+      <c r="E15" t="inlineStr"/>
       <c r="F15" t="inlineStr">
         <is>
           <t>Yes</t>
         </is>
       </c>
-      <c r="G15" t="inlineStr">
-        <is>
-          <t>Yes</t>
-        </is>
-      </c>
+      <c r="G15" t="inlineStr"/>
       <c r="H15" t="inlineStr">
         <is>
           <t>Yes</t>
@@ -1022,55 +1010,75 @@
       <c r="I15" t="inlineStr"/>
       <c r="J15" t="inlineStr"/>
       <c r="K15" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="L15" t="inlineStr"/>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>Colby Moon</t>
+          <t>Ben Berryhill</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>Yes</t>
-        </is>
-      </c>
-      <c r="C16" t="inlineStr"/>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="C16" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
       <c r="D16" t="inlineStr">
         <is>
           <t>Yes</t>
         </is>
       </c>
-      <c r="E16" t="inlineStr"/>
+      <c r="E16" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
       <c r="F16" t="inlineStr">
         <is>
           <t>Yes</t>
         </is>
       </c>
-      <c r="G16" t="inlineStr"/>
+      <c r="G16" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
       <c r="H16" t="inlineStr">
         <is>
-          <t>Yes</t>
+          <t>No</t>
         </is>
       </c>
       <c r="I16" t="inlineStr"/>
-      <c r="J16" t="inlineStr"/>
+      <c r="J16" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
       <c r="K16" t="n">
-        <v>3</v>
-      </c>
-      <c r="L16" t="inlineStr"/>
+        <v>4</v>
+      </c>
+      <c r="L16" t="inlineStr">
+        <is>
+          <t>08/07/2025-08/13/2025; 08/23/2025-08/30/2025</t>
+        </is>
+      </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>Ben Berryhill</t>
+          <t>Dean Mecham</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Yes</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
@@ -1095,33 +1103,25 @@
       </c>
       <c r="G17" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Yes</t>
         </is>
       </c>
       <c r="H17" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Yes</t>
         </is>
       </c>
       <c r="I17" t="inlineStr"/>
-      <c r="J17" t="inlineStr">
-        <is>
-          <t>Yes</t>
-        </is>
-      </c>
+      <c r="J17" t="inlineStr"/>
       <c r="K17" t="n">
         <v>4</v>
       </c>
-      <c r="L17" t="inlineStr">
-        <is>
-          <t>08/07/2025-08/13/2025; 08/23/2025-08/30/2025</t>
-        </is>
-      </c>
+      <c r="L17" t="inlineStr"/>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>Dean Mecham</t>
+          <t>Shawn Cross</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
@@ -1129,11 +1129,7 @@
           <t>Yes</t>
         </is>
       </c>
-      <c r="C18" t="inlineStr">
-        <is>
-          <t>Yes</t>
-        </is>
-      </c>
+      <c r="C18" t="inlineStr"/>
       <c r="D18" t="inlineStr">
         <is>
           <t>Yes</t>
@@ -1144,23 +1140,19 @@
           <t>Yes</t>
         </is>
       </c>
-      <c r="F18" t="inlineStr">
-        <is>
-          <t>Yes</t>
-        </is>
-      </c>
-      <c r="G18" t="inlineStr">
-        <is>
-          <t>Yes</t>
-        </is>
-      </c>
+      <c r="F18" t="inlineStr"/>
+      <c r="G18" t="inlineStr"/>
       <c r="H18" t="inlineStr">
         <is>
           <t>Yes</t>
         </is>
       </c>
       <c r="I18" t="inlineStr"/>
-      <c r="J18" t="inlineStr"/>
+      <c r="J18" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
       <c r="K18" t="n">
         <v>4</v>
       </c>
@@ -1169,7 +1161,7 @@
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>Shawn Cross</t>
+          <t>Tawai Finlayson</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
@@ -1178,17 +1170,17 @@
         </is>
       </c>
       <c r="C19" t="inlineStr"/>
-      <c r="D19" t="inlineStr">
-        <is>
-          <t>Yes</t>
-        </is>
-      </c>
+      <c r="D19" t="inlineStr"/>
       <c r="E19" t="inlineStr">
         <is>
           <t>Yes</t>
         </is>
       </c>
-      <c r="F19" t="inlineStr"/>
+      <c r="F19" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
       <c r="G19" t="inlineStr"/>
       <c r="H19" t="inlineStr">
         <is>
@@ -1209,7 +1201,7 @@
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>Tawai Finlayson</t>
+          <t>Philip Caputo</t>
         </is>
       </c>
       <c r="B20" t="inlineStr">
@@ -1217,24 +1209,24 @@
           <t>Yes</t>
         </is>
       </c>
-      <c r="C20" t="inlineStr"/>
+      <c r="C20" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
       <c r="D20" t="inlineStr"/>
-      <c r="E20" t="inlineStr">
-        <is>
-          <t>Yes</t>
-        </is>
-      </c>
+      <c r="E20" t="inlineStr"/>
       <c r="F20" t="inlineStr">
         <is>
           <t>Yes</t>
         </is>
       </c>
-      <c r="G20" t="inlineStr"/>
-      <c r="H20" t="inlineStr">
-        <is>
-          <t>Yes</t>
-        </is>
-      </c>
+      <c r="G20" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="H20" t="inlineStr"/>
       <c r="I20" t="inlineStr"/>
       <c r="J20" t="inlineStr">
         <is>
@@ -1249,38 +1241,18 @@
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>Philip Caputo</t>
-        </is>
-      </c>
-      <c r="B21" t="inlineStr">
-        <is>
-          <t>Yes</t>
-        </is>
-      </c>
-      <c r="C21" t="inlineStr">
-        <is>
-          <t>Yes</t>
-        </is>
-      </c>
+          <t>Rebe Flores</t>
+        </is>
+      </c>
+      <c r="B21" t="inlineStr"/>
+      <c r="C21" t="inlineStr"/>
       <c r="D21" t="inlineStr"/>
       <c r="E21" t="inlineStr"/>
-      <c r="F21" t="inlineStr">
-        <is>
-          <t>Yes</t>
-        </is>
-      </c>
-      <c r="G21" t="inlineStr">
-        <is>
-          <t>Yes</t>
-        </is>
-      </c>
+      <c r="F21" t="inlineStr"/>
+      <c r="G21" t="inlineStr"/>
       <c r="H21" t="inlineStr"/>
       <c r="I21" t="inlineStr"/>
-      <c r="J21" t="inlineStr">
-        <is>
-          <t>Yes</t>
-        </is>
-      </c>
+      <c r="J21" t="inlineStr"/>
       <c r="K21" t="n">
         <v>4</v>
       </c>
@@ -1289,31 +1261,55 @@
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>Rebe Flores</t>
+          <t>Jerin Palmer</t>
         </is>
       </c>
       <c r="B22" t="inlineStr"/>
       <c r="C22" t="inlineStr"/>
-      <c r="D22" t="inlineStr"/>
-      <c r="E22" t="inlineStr"/>
-      <c r="F22" t="inlineStr"/>
+      <c r="D22" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="E22" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="F22" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
       <c r="G22" t="inlineStr"/>
       <c r="H22" t="inlineStr"/>
       <c r="I22" t="inlineStr"/>
-      <c r="J22" t="inlineStr"/>
+      <c r="J22" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
       <c r="K22" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="L22" t="inlineStr"/>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>Jerin Palmer</t>
-        </is>
-      </c>
-      <c r="B23" t="inlineStr"/>
-      <c r="C23" t="inlineStr"/>
+          <t>Nathaniel Spice</t>
+        </is>
+      </c>
+      <c r="B23" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="C23" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
       <c r="D23" t="inlineStr">
         <is>
           <t>Yes</t>
@@ -1324,11 +1320,7 @@
           <t>Yes</t>
         </is>
       </c>
-      <c r="F23" t="inlineStr">
-        <is>
-          <t>Yes</t>
-        </is>
-      </c>
+      <c r="F23" t="inlineStr"/>
       <c r="G23" t="inlineStr"/>
       <c r="H23" t="inlineStr"/>
       <c r="I23" t="inlineStr"/>
@@ -1338,21 +1330,17 @@
         </is>
       </c>
       <c r="K23" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="L23" t="inlineStr"/>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>Nathaniel Spice</t>
-        </is>
-      </c>
-      <c r="B24" t="inlineStr">
-        <is>
-          <t>Yes</t>
-        </is>
-      </c>
+          <t>Charlie Dopp</t>
+        </is>
+      </c>
+      <c r="B24" t="inlineStr"/>
       <c r="C24" t="inlineStr">
         <is>
           <t>Yes</t>
@@ -1368,15 +1356,23 @@
           <t>Yes</t>
         </is>
       </c>
-      <c r="F24" t="inlineStr"/>
-      <c r="G24" t="inlineStr"/>
-      <c r="H24" t="inlineStr"/>
+      <c r="F24" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="G24" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="H24" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
       <c r="I24" t="inlineStr"/>
-      <c r="J24" t="inlineStr">
-        <is>
-          <t>Yes</t>
-        </is>
-      </c>
+      <c r="J24" t="inlineStr"/>
       <c r="K24" t="n">
         <v>4</v>
       </c>
@@ -1385,7 +1381,7 @@
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>Charlie Dopp</t>
+          <t>John Dean</t>
         </is>
       </c>
       <c r="B25" t="inlineStr"/>
@@ -1399,16 +1395,8 @@
           <t>Yes</t>
         </is>
       </c>
-      <c r="E25" t="inlineStr">
-        <is>
-          <t>Yes</t>
-        </is>
-      </c>
-      <c r="F25" t="inlineStr">
-        <is>
-          <t>Yes</t>
-        </is>
-      </c>
+      <c r="E25" t="inlineStr"/>
+      <c r="F25" t="inlineStr"/>
       <c r="G25" t="inlineStr">
         <is>
           <t>Yes</t>
@@ -1420,7 +1408,11 @@
         </is>
       </c>
       <c r="I25" t="inlineStr"/>
-      <c r="J25" t="inlineStr"/>
+      <c r="J25" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
       <c r="K25" t="n">
         <v>4</v>
       </c>
@@ -1429,38 +1421,18 @@
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>John Dean</t>
+          <t>Weston Hamilton</t>
         </is>
       </c>
       <c r="B26" t="inlineStr"/>
-      <c r="C26" t="inlineStr">
-        <is>
-          <t>Yes</t>
-        </is>
-      </c>
-      <c r="D26" t="inlineStr">
-        <is>
-          <t>Yes</t>
-        </is>
-      </c>
+      <c r="C26" t="inlineStr"/>
+      <c r="D26" t="inlineStr"/>
       <c r="E26" t="inlineStr"/>
       <c r="F26" t="inlineStr"/>
-      <c r="G26" t="inlineStr">
-        <is>
-          <t>Yes</t>
-        </is>
-      </c>
-      <c r="H26" t="inlineStr">
-        <is>
-          <t>Yes</t>
-        </is>
-      </c>
+      <c r="G26" t="inlineStr"/>
+      <c r="H26" t="inlineStr"/>
       <c r="I26" t="inlineStr"/>
-      <c r="J26" t="inlineStr">
-        <is>
-          <t>Yes</t>
-        </is>
-      </c>
+      <c r="J26" t="inlineStr"/>
       <c r="K26" t="n">
         <v>4</v>
       </c>
@@ -1469,18 +1441,38 @@
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>Weston Hamilton</t>
+          <t>Tyler Freeze</t>
         </is>
       </c>
       <c r="B27" t="inlineStr"/>
-      <c r="C27" t="inlineStr"/>
+      <c r="C27" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
       <c r="D27" t="inlineStr"/>
-      <c r="E27" t="inlineStr"/>
+      <c r="E27" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
       <c r="F27" t="inlineStr"/>
-      <c r="G27" t="inlineStr"/>
-      <c r="H27" t="inlineStr"/>
+      <c r="G27" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="H27" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
       <c r="I27" t="inlineStr"/>
-      <c r="J27" t="inlineStr"/>
+      <c r="J27" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
       <c r="K27" t="n">
         <v>4</v>
       </c>
@@ -1489,7 +1481,7 @@
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>Tyler Freeze</t>
+          <t>Michael Dean</t>
         </is>
       </c>
       <c r="B28" t="inlineStr"/>
@@ -1498,12 +1490,12 @@
           <t>Yes</t>
         </is>
       </c>
-      <c r="D28" t="inlineStr"/>
-      <c r="E28" t="inlineStr">
-        <is>
-          <t>Yes</t>
-        </is>
-      </c>
+      <c r="D28" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="E28" t="inlineStr"/>
       <c r="F28" t="inlineStr"/>
       <c r="G28" t="inlineStr">
         <is>
@@ -1529,21 +1521,21 @@
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>Michael Dean</t>
+          <t>Robert Prudhomme</t>
         </is>
       </c>
       <c r="B29" t="inlineStr"/>
-      <c r="C29" t="inlineStr">
-        <is>
-          <t>Yes</t>
-        </is>
-      </c>
+      <c r="C29" t="inlineStr"/>
       <c r="D29" t="inlineStr">
         <is>
           <t>Yes</t>
         </is>
       </c>
-      <c r="E29" t="inlineStr"/>
+      <c r="E29" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
       <c r="F29" t="inlineStr"/>
       <c r="G29" t="inlineStr">
         <is>
@@ -1569,38 +1561,18 @@
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>Robert Prudhomme</t>
+          <t>Tyler Walker</t>
         </is>
       </c>
       <c r="B30" t="inlineStr"/>
       <c r="C30" t="inlineStr"/>
-      <c r="D30" t="inlineStr">
-        <is>
-          <t>Yes</t>
-        </is>
-      </c>
-      <c r="E30" t="inlineStr">
-        <is>
-          <t>Yes</t>
-        </is>
-      </c>
+      <c r="D30" t="inlineStr"/>
+      <c r="E30" t="inlineStr"/>
       <c r="F30" t="inlineStr"/>
-      <c r="G30" t="inlineStr">
-        <is>
-          <t>Yes</t>
-        </is>
-      </c>
-      <c r="H30" t="inlineStr">
-        <is>
-          <t>Yes</t>
-        </is>
-      </c>
+      <c r="G30" t="inlineStr"/>
+      <c r="H30" t="inlineStr"/>
       <c r="I30" t="inlineStr"/>
-      <c r="J30" t="inlineStr">
-        <is>
-          <t>Yes</t>
-        </is>
-      </c>
+      <c r="J30" t="inlineStr"/>
       <c r="K30" t="n">
         <v>4</v>
       </c>
@@ -1609,18 +1581,34 @@
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>Tyler Walker</t>
+          <t>Houston Griffith</t>
         </is>
       </c>
       <c r="B31" t="inlineStr"/>
       <c r="C31" t="inlineStr"/>
-      <c r="D31" t="inlineStr"/>
+      <c r="D31" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
       <c r="E31" t="inlineStr"/>
-      <c r="F31" t="inlineStr"/>
+      <c r="F31" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
       <c r="G31" t="inlineStr"/>
-      <c r="H31" t="inlineStr"/>
+      <c r="H31" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
       <c r="I31" t="inlineStr"/>
-      <c r="J31" t="inlineStr"/>
+      <c r="J31" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
       <c r="K31" t="n">
         <v>4</v>
       </c>
@@ -1629,34 +1617,46 @@
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>Houston Griffith</t>
-        </is>
-      </c>
-      <c r="B32" t="inlineStr"/>
-      <c r="C32" t="inlineStr"/>
+          <t>Jerrin Foster</t>
+        </is>
+      </c>
+      <c r="B32" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="C32" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
       <c r="D32" t="inlineStr">
         <is>
           <t>Yes</t>
         </is>
       </c>
-      <c r="E32" t="inlineStr"/>
+      <c r="E32" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
       <c r="F32" t="inlineStr">
         <is>
           <t>Yes</t>
         </is>
       </c>
-      <c r="G32" t="inlineStr"/>
+      <c r="G32" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
       <c r="H32" t="inlineStr">
         <is>
           <t>Yes</t>
         </is>
       </c>
       <c r="I32" t="inlineStr"/>
-      <c r="J32" t="inlineStr">
-        <is>
-          <t>Yes</t>
-        </is>
-      </c>
+      <c r="J32" t="inlineStr"/>
       <c r="K32" t="n">
         <v>4</v>
       </c>
@@ -1665,7 +1665,7 @@
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>Jerrin Foster</t>
+          <t>Connor Lund</t>
         </is>
       </c>
       <c r="B33" t="inlineStr">
@@ -1673,21 +1673,13 @@
           <t>Yes</t>
         </is>
       </c>
-      <c r="C33" t="inlineStr">
-        <is>
-          <t>Yes</t>
-        </is>
-      </c>
+      <c r="C33" t="inlineStr"/>
       <c r="D33" t="inlineStr">
         <is>
           <t>Yes</t>
         </is>
       </c>
-      <c r="E33" t="inlineStr">
-        <is>
-          <t>Yes</t>
-        </is>
-      </c>
+      <c r="E33" t="inlineStr"/>
       <c r="F33" t="inlineStr">
         <is>
           <t>Yes</t>
@@ -1706,33 +1698,25 @@
       <c r="I33" t="inlineStr"/>
       <c r="J33" t="inlineStr"/>
       <c r="K33" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="L33" t="inlineStr"/>
     </row>
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t>Connor Lund</t>
-        </is>
-      </c>
-      <c r="B34" t="inlineStr">
-        <is>
-          <t>Yes</t>
-        </is>
-      </c>
+          <t>Roberto Guevara</t>
+        </is>
+      </c>
+      <c r="B34" t="inlineStr"/>
       <c r="C34" t="inlineStr"/>
-      <c r="D34" t="inlineStr">
-        <is>
-          <t>Yes</t>
-        </is>
-      </c>
-      <c r="E34" t="inlineStr"/>
-      <c r="F34" t="inlineStr">
-        <is>
-          <t>Yes</t>
-        </is>
-      </c>
+      <c r="D34" t="inlineStr"/>
+      <c r="E34" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="F34" t="inlineStr"/>
       <c r="G34" t="inlineStr">
         <is>
           <t>Yes</t>
@@ -1744,27 +1728,47 @@
         </is>
       </c>
       <c r="I34" t="inlineStr"/>
-      <c r="J34" t="inlineStr"/>
+      <c r="J34" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
       <c r="K34" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="L34" t="inlineStr"/>
     </row>
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>Roberto Guevara</t>
-        </is>
-      </c>
-      <c r="B35" t="inlineStr"/>
-      <c r="C35" t="inlineStr"/>
-      <c r="D35" t="inlineStr"/>
+          <t>Seth Heilesen</t>
+        </is>
+      </c>
+      <c r="B35" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="C35" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="D35" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
       <c r="E35" t="inlineStr">
         <is>
           <t>Yes</t>
         </is>
       </c>
-      <c r="F35" t="inlineStr"/>
+      <c r="F35" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
       <c r="G35" t="inlineStr">
         <is>
           <t>Yes</t>
@@ -1776,20 +1780,16 @@
         </is>
       </c>
       <c r="I35" t="inlineStr"/>
-      <c r="J35" t="inlineStr">
-        <is>
-          <t>Yes</t>
-        </is>
-      </c>
+      <c r="J35" t="inlineStr"/>
       <c r="K35" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="L35" t="inlineStr"/>
     </row>
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
-          <t>Seth Heilesen</t>
+          <t>Arianna Jenkins</t>
         </is>
       </c>
       <c r="B36" t="inlineStr">
@@ -1797,26 +1797,14 @@
           <t>Yes</t>
         </is>
       </c>
-      <c r="C36" t="inlineStr">
-        <is>
-          <t>Yes</t>
-        </is>
-      </c>
-      <c r="D36" t="inlineStr">
-        <is>
-          <t>Yes</t>
-        </is>
-      </c>
+      <c r="C36" t="inlineStr"/>
+      <c r="D36" t="inlineStr"/>
       <c r="E36" t="inlineStr">
         <is>
           <t>Yes</t>
         </is>
       </c>
-      <c r="F36" t="inlineStr">
-        <is>
-          <t>Yes</t>
-        </is>
-      </c>
+      <c r="F36" t="inlineStr"/>
       <c r="G36" t="inlineStr">
         <is>
           <t>Yes</t>
@@ -1830,14 +1818,14 @@
       <c r="I36" t="inlineStr"/>
       <c r="J36" t="inlineStr"/>
       <c r="K36" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="L36" t="inlineStr"/>
     </row>
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t>Arianna Jenkins</t>
+          <t>Amanda Rodriguez</t>
         </is>
       </c>
       <c r="B37" t="inlineStr">
@@ -1845,7 +1833,11 @@
           <t>Yes</t>
         </is>
       </c>
-      <c r="C37" t="inlineStr"/>
+      <c r="C37" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
       <c r="D37" t="inlineStr"/>
       <c r="E37" t="inlineStr">
         <is>
@@ -1858,11 +1850,7 @@
           <t>Yes</t>
         </is>
       </c>
-      <c r="H37" t="inlineStr">
-        <is>
-          <t>Yes</t>
-        </is>
-      </c>
+      <c r="H37" t="inlineStr"/>
       <c r="I37" t="inlineStr"/>
       <c r="J37" t="inlineStr"/>
       <c r="K37" t="n">
@@ -1873,7 +1861,7 @@
     <row r="38">
       <c r="A38" t="inlineStr">
         <is>
-          <t>Amanda Rodriguez</t>
+          <t>Jasmine Girard-Posey</t>
         </is>
       </c>
       <c r="B38" t="inlineStr">
@@ -1881,26 +1869,26 @@
           <t>Yes</t>
         </is>
       </c>
-      <c r="C38" t="inlineStr">
-        <is>
-          <t>Yes</t>
-        </is>
-      </c>
+      <c r="C38" t="inlineStr"/>
       <c r="D38" t="inlineStr"/>
       <c r="E38" t="inlineStr">
         <is>
           <t>Yes</t>
         </is>
       </c>
-      <c r="F38" t="inlineStr"/>
-      <c r="G38" t="inlineStr">
-        <is>
-          <t>Yes</t>
-        </is>
-      </c>
+      <c r="F38" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="G38" t="inlineStr"/>
       <c r="H38" t="inlineStr"/>
       <c r="I38" t="inlineStr"/>
-      <c r="J38" t="inlineStr"/>
+      <c r="J38" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
       <c r="K38" t="n">
         <v>4</v>
       </c>
@@ -1909,7 +1897,7 @@
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t>Jasmine Girard-Posey</t>
+          <t>Devin Butler</t>
         </is>
       </c>
       <c r="B39" t="inlineStr">
@@ -1917,18 +1905,18 @@
           <t>Yes</t>
         </is>
       </c>
-      <c r="C39" t="inlineStr"/>
-      <c r="D39" t="inlineStr"/>
-      <c r="E39" t="inlineStr">
-        <is>
-          <t>Yes</t>
-        </is>
-      </c>
-      <c r="F39" t="inlineStr">
-        <is>
-          <t>Yes</t>
-        </is>
-      </c>
+      <c r="C39" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="D39" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="E39" t="inlineStr"/>
+      <c r="F39" t="inlineStr"/>
       <c r="G39" t="inlineStr"/>
       <c r="H39" t="inlineStr"/>
       <c r="I39" t="inlineStr"/>
@@ -1938,14 +1926,14 @@
         </is>
       </c>
       <c r="K39" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="L39" t="inlineStr"/>
     </row>
     <row r="40">
       <c r="A40" t="inlineStr">
         <is>
-          <t>Devin Butler</t>
+          <t>Nancy Girard</t>
         </is>
       </c>
       <c r="B40" t="inlineStr">
@@ -1963,25 +1951,37 @@
           <t>Yes</t>
         </is>
       </c>
-      <c r="E40" t="inlineStr"/>
-      <c r="F40" t="inlineStr"/>
-      <c r="G40" t="inlineStr"/>
-      <c r="H40" t="inlineStr"/>
+      <c r="E40" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="F40" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="G40" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="H40" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
       <c r="I40" t="inlineStr"/>
-      <c r="J40" t="inlineStr">
-        <is>
-          <t>Yes</t>
-        </is>
-      </c>
+      <c r="J40" t="inlineStr"/>
       <c r="K40" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="L40" t="inlineStr"/>
     </row>
     <row r="41">
       <c r="A41" t="inlineStr">
         <is>
-          <t>Nancy Girard</t>
+          <t>Aaron Parker</t>
         </is>
       </c>
       <c r="B41" t="inlineStr">
@@ -2029,7 +2029,7 @@
     <row r="42">
       <c r="A42" t="inlineStr">
         <is>
-          <t>Aaron Parker</t>
+          <t>Alex Lopez</t>
         </is>
       </c>
       <c r="B42" t="inlineStr">
@@ -2077,19 +2077,11 @@
     <row r="43">
       <c r="A43" t="inlineStr">
         <is>
-          <t>Alex Lopez</t>
-        </is>
-      </c>
-      <c r="B43" t="inlineStr">
-        <is>
-          <t>Yes</t>
-        </is>
-      </c>
-      <c r="C43" t="inlineStr">
-        <is>
-          <t>Yes</t>
-        </is>
-      </c>
+          <t>Jake Belt</t>
+        </is>
+      </c>
+      <c r="B43" t="inlineStr"/>
+      <c r="C43" t="inlineStr"/>
       <c r="D43" t="inlineStr">
         <is>
           <t>Yes</t>
@@ -2100,11 +2092,7 @@
           <t>Yes</t>
         </is>
       </c>
-      <c r="F43" t="inlineStr">
-        <is>
-          <t>Yes</t>
-        </is>
-      </c>
+      <c r="F43" t="inlineStr"/>
       <c r="G43" t="inlineStr">
         <is>
           <t>Yes</t>
@@ -2125,32 +2113,24 @@
     <row r="44">
       <c r="A44" t="inlineStr">
         <is>
-          <t>Jake Belt</t>
+          <t>Tyler Mautz</t>
         </is>
       </c>
       <c r="B44" t="inlineStr"/>
-      <c r="C44" t="inlineStr"/>
+      <c r="C44" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
       <c r="D44" t="inlineStr">
         <is>
           <t>Yes</t>
         </is>
       </c>
-      <c r="E44" t="inlineStr">
-        <is>
-          <t>Yes</t>
-        </is>
-      </c>
+      <c r="E44" t="inlineStr"/>
       <c r="F44" t="inlineStr"/>
-      <c r="G44" t="inlineStr">
-        <is>
-          <t>Yes</t>
-        </is>
-      </c>
-      <c r="H44" t="inlineStr">
-        <is>
-          <t>Yes</t>
-        </is>
-      </c>
+      <c r="G44" t="inlineStr"/>
+      <c r="H44" t="inlineStr"/>
       <c r="I44" t="inlineStr"/>
       <c r="J44" t="inlineStr"/>
       <c r="K44" t="n">
@@ -2161,20 +2141,12 @@
     <row r="45">
       <c r="A45" t="inlineStr">
         <is>
-          <t>Tyler Mautz</t>
+          <t>Travis Moffat</t>
         </is>
       </c>
       <c r="B45" t="inlineStr"/>
-      <c r="C45" t="inlineStr">
-        <is>
-          <t>Yes</t>
-        </is>
-      </c>
-      <c r="D45" t="inlineStr">
-        <is>
-          <t>Yes</t>
-        </is>
-      </c>
+      <c r="C45" t="inlineStr"/>
+      <c r="D45" t="inlineStr"/>
       <c r="E45" t="inlineStr"/>
       <c r="F45" t="inlineStr"/>
       <c r="G45" t="inlineStr"/>
@@ -2189,27 +2161,43 @@
     <row r="46">
       <c r="A46" t="inlineStr">
         <is>
-          <t>Travis Moffat</t>
-        </is>
-      </c>
-      <c r="B46" t="inlineStr"/>
-      <c r="C46" t="inlineStr"/>
-      <c r="D46" t="inlineStr"/>
-      <c r="E46" t="inlineStr"/>
+          <t>Evan Doman</t>
+        </is>
+      </c>
+      <c r="B46" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="C46" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="D46" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="E46" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
       <c r="F46" t="inlineStr"/>
       <c r="G46" t="inlineStr"/>
       <c r="H46" t="inlineStr"/>
       <c r="I46" t="inlineStr"/>
       <c r="J46" t="inlineStr"/>
       <c r="K46" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="L46" t="inlineStr"/>
     </row>
     <row r="47">
       <c r="A47" t="inlineStr">
         <is>
-          <t>Evan Doman</t>
+          <t>Ethan McCray</t>
         </is>
       </c>
       <c r="B47" t="inlineStr">
@@ -2232,20 +2220,32 @@
           <t>Yes</t>
         </is>
       </c>
-      <c r="F47" t="inlineStr"/>
-      <c r="G47" t="inlineStr"/>
-      <c r="H47" t="inlineStr"/>
+      <c r="F47" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="G47" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="H47" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
       <c r="I47" t="inlineStr"/>
       <c r="J47" t="inlineStr"/>
       <c r="K47" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="L47" t="inlineStr"/>
     </row>
     <row r="48">
       <c r="A48" t="inlineStr">
         <is>
-          <t>Ethan McCray</t>
+          <t>Marcus Gibby</t>
         </is>
       </c>
       <c r="B48" t="inlineStr">
@@ -2253,11 +2253,7 @@
           <t>Yes</t>
         </is>
       </c>
-      <c r="C48" t="inlineStr">
-        <is>
-          <t>Yes</t>
-        </is>
-      </c>
+      <c r="C48" t="inlineStr"/>
       <c r="D48" t="inlineStr">
         <is>
           <t>Yes</t>
@@ -2273,11 +2269,7 @@
           <t>Yes</t>
         </is>
       </c>
-      <c r="G48" t="inlineStr">
-        <is>
-          <t>Yes</t>
-        </is>
-      </c>
+      <c r="G48" t="inlineStr"/>
       <c r="H48" t="inlineStr">
         <is>
           <t>Yes</t>
@@ -2286,14 +2278,14 @@
       <c r="I48" t="inlineStr"/>
       <c r="J48" t="inlineStr"/>
       <c r="K48" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="L48" t="inlineStr"/>
     </row>
     <row r="49">
       <c r="A49" t="inlineStr">
         <is>
-          <t>Marcus Gibby</t>
+          <t>Jayson Burke</t>
         </is>
       </c>
       <c r="B49" t="inlineStr">
@@ -2301,7 +2293,11 @@
           <t>Yes</t>
         </is>
       </c>
-      <c r="C49" t="inlineStr"/>
+      <c r="C49" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
       <c r="D49" t="inlineStr">
         <is>
           <t>Yes</t>
@@ -2317,7 +2313,11 @@
           <t>Yes</t>
         </is>
       </c>
-      <c r="G49" t="inlineStr"/>
+      <c r="G49" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
       <c r="H49" t="inlineStr">
         <is>
           <t>Yes</t>
@@ -2326,14 +2326,14 @@
       <c r="I49" t="inlineStr"/>
       <c r="J49" t="inlineStr"/>
       <c r="K49" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="L49" t="inlineStr"/>
     </row>
     <row r="50">
       <c r="A50" t="inlineStr">
         <is>
-          <t>Jayson Burke</t>
+          <t>Sarin Thorn</t>
         </is>
       </c>
       <c r="B50" t="inlineStr">
@@ -2341,38 +2341,22 @@
           <t>Yes</t>
         </is>
       </c>
-      <c r="C50" t="inlineStr">
-        <is>
-          <t>Yes</t>
-        </is>
-      </c>
-      <c r="D50" t="inlineStr">
-        <is>
-          <t>Yes</t>
-        </is>
-      </c>
-      <c r="E50" t="inlineStr">
-        <is>
-          <t>Yes</t>
-        </is>
-      </c>
-      <c r="F50" t="inlineStr">
-        <is>
-          <t>Yes</t>
-        </is>
-      </c>
-      <c r="G50" t="inlineStr">
-        <is>
-          <t>Yes</t>
-        </is>
-      </c>
+      <c r="C50" t="inlineStr"/>
+      <c r="D50" t="inlineStr"/>
+      <c r="E50" t="inlineStr"/>
+      <c r="F50" t="inlineStr"/>
+      <c r="G50" t="inlineStr"/>
       <c r="H50" t="inlineStr">
         <is>
           <t>Yes</t>
         </is>
       </c>
       <c r="I50" t="inlineStr"/>
-      <c r="J50" t="inlineStr"/>
+      <c r="J50" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
       <c r="K50" t="n">
         <v>4</v>
       </c>
@@ -2381,30 +2365,18 @@
     <row r="51">
       <c r="A51" t="inlineStr">
         <is>
-          <t>Sarin Thorn</t>
-        </is>
-      </c>
-      <c r="B51" t="inlineStr">
-        <is>
-          <t>Yes</t>
-        </is>
-      </c>
+          <t>David Gardner</t>
+        </is>
+      </c>
+      <c r="B51" t="inlineStr"/>
       <c r="C51" t="inlineStr"/>
       <c r="D51" t="inlineStr"/>
       <c r="E51" t="inlineStr"/>
       <c r="F51" t="inlineStr"/>
       <c r="G51" t="inlineStr"/>
-      <c r="H51" t="inlineStr">
-        <is>
-          <t>Yes</t>
-        </is>
-      </c>
+      <c r="H51" t="inlineStr"/>
       <c r="I51" t="inlineStr"/>
-      <c r="J51" t="inlineStr">
-        <is>
-          <t>Yes</t>
-        </is>
-      </c>
+      <c r="J51" t="inlineStr"/>
       <c r="K51" t="n">
         <v>4</v>
       </c>
@@ -2413,7 +2385,7 @@
     <row r="52">
       <c r="A52" t="inlineStr">
         <is>
-          <t>David Gardner</t>
+          <t>Robin Larsen</t>
         </is>
       </c>
       <c r="B52" t="inlineStr"/>
@@ -2433,18 +2405,34 @@
     <row r="53">
       <c r="A53" t="inlineStr">
         <is>
-          <t>Robin Larsen</t>
-        </is>
-      </c>
-      <c r="B53" t="inlineStr"/>
-      <c r="C53" t="inlineStr"/>
+          <t>Cortez Gee</t>
+        </is>
+      </c>
+      <c r="B53" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="C53" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
       <c r="D53" t="inlineStr"/>
       <c r="E53" t="inlineStr"/>
-      <c r="F53" t="inlineStr"/>
+      <c r="F53" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
       <c r="G53" t="inlineStr"/>
       <c r="H53" t="inlineStr"/>
       <c r="I53" t="inlineStr"/>
-      <c r="J53" t="inlineStr"/>
+      <c r="J53" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
       <c r="K53" t="n">
         <v>4</v>
       </c>
@@ -2453,34 +2441,18 @@
     <row r="54">
       <c r="A54" t="inlineStr">
         <is>
-          <t>Cortez Gee</t>
-        </is>
-      </c>
-      <c r="B54" t="inlineStr">
-        <is>
-          <t>Yes</t>
-        </is>
-      </c>
-      <c r="C54" t="inlineStr">
-        <is>
-          <t>Yes</t>
-        </is>
-      </c>
+          <t>Dianne McCann</t>
+        </is>
+      </c>
+      <c r="B54" t="inlineStr"/>
+      <c r="C54" t="inlineStr"/>
       <c r="D54" t="inlineStr"/>
       <c r="E54" t="inlineStr"/>
-      <c r="F54" t="inlineStr">
-        <is>
-          <t>Yes</t>
-        </is>
-      </c>
+      <c r="F54" t="inlineStr"/>
       <c r="G54" t="inlineStr"/>
       <c r="H54" t="inlineStr"/>
       <c r="I54" t="inlineStr"/>
-      <c r="J54" t="inlineStr">
-        <is>
-          <t>Yes</t>
-        </is>
-      </c>
+      <c r="J54" t="inlineStr"/>
       <c r="K54" t="n">
         <v>4</v>
       </c>
@@ -2489,18 +2461,38 @@
     <row r="55">
       <c r="A55" t="inlineStr">
         <is>
-          <t>Dianne McCann</t>
+          <t>Diana Islas</t>
         </is>
       </c>
       <c r="B55" t="inlineStr"/>
-      <c r="C55" t="inlineStr"/>
-      <c r="D55" t="inlineStr"/>
+      <c r="C55" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="D55" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
       <c r="E55" t="inlineStr"/>
       <c r="F55" t="inlineStr"/>
-      <c r="G55" t="inlineStr"/>
-      <c r="H55" t="inlineStr"/>
+      <c r="G55" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="H55" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
       <c r="I55" t="inlineStr"/>
-      <c r="J55" t="inlineStr"/>
+      <c r="J55" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
       <c r="K55" t="n">
         <v>4</v>
       </c>
@@ -2509,38 +2501,18 @@
     <row r="56">
       <c r="A56" t="inlineStr">
         <is>
-          <t>Diana Islas</t>
+          <t>Keenan Karratti</t>
         </is>
       </c>
       <c r="B56" t="inlineStr"/>
-      <c r="C56" t="inlineStr">
-        <is>
-          <t>Yes</t>
-        </is>
-      </c>
-      <c r="D56" t="inlineStr">
-        <is>
-          <t>Yes</t>
-        </is>
-      </c>
+      <c r="C56" t="inlineStr"/>
+      <c r="D56" t="inlineStr"/>
       <c r="E56" t="inlineStr"/>
       <c r="F56" t="inlineStr"/>
-      <c r="G56" t="inlineStr">
-        <is>
-          <t>Yes</t>
-        </is>
-      </c>
-      <c r="H56" t="inlineStr">
-        <is>
-          <t>Yes</t>
-        </is>
-      </c>
+      <c r="G56" t="inlineStr"/>
+      <c r="H56" t="inlineStr"/>
       <c r="I56" t="inlineStr"/>
-      <c r="J56" t="inlineStr">
-        <is>
-          <t>Yes</t>
-        </is>
-      </c>
+      <c r="J56" t="inlineStr"/>
       <c r="K56" t="n">
         <v>4</v>
       </c>
@@ -2549,18 +2521,34 @@
     <row r="57">
       <c r="A57" t="inlineStr">
         <is>
-          <t>Keenan Karratti</t>
-        </is>
-      </c>
-      <c r="B57" t="inlineStr"/>
+          <t>Kalen Avila</t>
+        </is>
+      </c>
+      <c r="B57" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
       <c r="C57" t="inlineStr"/>
-      <c r="D57" t="inlineStr"/>
+      <c r="D57" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
       <c r="E57" t="inlineStr"/>
-      <c r="F57" t="inlineStr"/>
+      <c r="F57" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
       <c r="G57" t="inlineStr"/>
       <c r="H57" t="inlineStr"/>
       <c r="I57" t="inlineStr"/>
-      <c r="J57" t="inlineStr"/>
+      <c r="J57" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
       <c r="K57" t="n">
         <v>4</v>
       </c>
@@ -2569,54 +2557,66 @@
     <row r="58">
       <c r="A58" t="inlineStr">
         <is>
-          <t>Kalen Avila</t>
-        </is>
-      </c>
-      <c r="B58" t="inlineStr">
-        <is>
-          <t>Yes</t>
-        </is>
-      </c>
-      <c r="C58" t="inlineStr"/>
-      <c r="D58" t="inlineStr">
-        <is>
-          <t>Yes</t>
-        </is>
-      </c>
+          <t>Brianna Graves</t>
+        </is>
+      </c>
+      <c r="B58" t="inlineStr"/>
+      <c r="C58" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="D58" t="inlineStr"/>
       <c r="E58" t="inlineStr"/>
-      <c r="F58" t="inlineStr">
-        <is>
-          <t>Yes</t>
-        </is>
-      </c>
-      <c r="G58" t="inlineStr"/>
-      <c r="H58" t="inlineStr"/>
+      <c r="F58" t="inlineStr"/>
+      <c r="G58" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="H58" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
       <c r="I58" t="inlineStr"/>
-      <c r="J58" t="inlineStr">
-        <is>
-          <t>Yes</t>
-        </is>
-      </c>
+      <c r="J58" t="inlineStr"/>
       <c r="K58" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="L58" t="inlineStr"/>
     </row>
     <row r="59">
       <c r="A59" t="inlineStr">
         <is>
-          <t>Brianna Graves</t>
-        </is>
-      </c>
-      <c r="B59" t="inlineStr"/>
+          <t>Jason Faux</t>
+        </is>
+      </c>
+      <c r="B59" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
       <c r="C59" t="inlineStr">
         <is>
           <t>Yes</t>
         </is>
       </c>
-      <c r="D59" t="inlineStr"/>
-      <c r="E59" t="inlineStr"/>
-      <c r="F59" t="inlineStr"/>
+      <c r="D59" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="E59" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="F59" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
       <c r="G59" t="inlineStr">
         <is>
           <t>Yes</t>
@@ -2630,21 +2630,17 @@
       <c r="I59" t="inlineStr"/>
       <c r="J59" t="inlineStr"/>
       <c r="K59" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="L59" t="inlineStr"/>
     </row>
     <row r="60">
       <c r="A60" t="inlineStr">
         <is>
-          <t>Jason Faux</t>
-        </is>
-      </c>
-      <c r="B60" t="inlineStr">
-        <is>
-          <t>Yes</t>
-        </is>
-      </c>
+          <t>Ethan Gilbert</t>
+        </is>
+      </c>
+      <c r="B60" t="inlineStr"/>
       <c r="C60" t="inlineStr">
         <is>
           <t>Yes</t>
@@ -2655,16 +2651,8 @@
           <t>Yes</t>
         </is>
       </c>
-      <c r="E60" t="inlineStr">
-        <is>
-          <t>Yes</t>
-        </is>
-      </c>
-      <c r="F60" t="inlineStr">
-        <is>
-          <t>Yes</t>
-        </is>
-      </c>
+      <c r="E60" t="inlineStr"/>
+      <c r="F60" t="inlineStr"/>
       <c r="G60" t="inlineStr">
         <is>
           <t>Yes</t>
@@ -2676,7 +2664,11 @@
         </is>
       </c>
       <c r="I60" t="inlineStr"/>
-      <c r="J60" t="inlineStr"/>
+      <c r="J60" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
       <c r="K60" t="n">
         <v>4</v>
       </c>
@@ -2685,7 +2677,7 @@
     <row r="61">
       <c r="A61" t="inlineStr">
         <is>
-          <t>Ethan Gilbert</t>
+          <t>Vincent Hancock</t>
         </is>
       </c>
       <c r="B61" t="inlineStr"/>
@@ -2725,27 +2717,19 @@
     <row r="62">
       <c r="A62" t="inlineStr">
         <is>
-          <t>Vincent Hancock</t>
-        </is>
-      </c>
-      <c r="B62" t="inlineStr"/>
-      <c r="C62" t="inlineStr">
-        <is>
-          <t>Yes</t>
-        </is>
-      </c>
-      <c r="D62" t="inlineStr">
-        <is>
-          <t>Yes</t>
-        </is>
-      </c>
+          <t>Brady Alvey</t>
+        </is>
+      </c>
+      <c r="B62" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="C62" t="inlineStr"/>
+      <c r="D62" t="inlineStr"/>
       <c r="E62" t="inlineStr"/>
       <c r="F62" t="inlineStr"/>
-      <c r="G62" t="inlineStr">
-        <is>
-          <t>Yes</t>
-        </is>
-      </c>
+      <c r="G62" t="inlineStr"/>
       <c r="H62" t="inlineStr">
         <is>
           <t>Yes</t>
@@ -2765,17 +2749,25 @@
     <row r="63">
       <c r="A63" t="inlineStr">
         <is>
-          <t>Brady Alvey</t>
-        </is>
-      </c>
-      <c r="B63" t="inlineStr">
-        <is>
-          <t>Yes</t>
-        </is>
-      </c>
-      <c r="C63" t="inlineStr"/>
-      <c r="D63" t="inlineStr"/>
-      <c r="E63" t="inlineStr"/>
+          <t>Jesus Reyes</t>
+        </is>
+      </c>
+      <c r="B63" t="inlineStr"/>
+      <c r="C63" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="D63" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="E63" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
       <c r="F63" t="inlineStr"/>
       <c r="G63" t="inlineStr"/>
       <c r="H63" t="inlineStr">
@@ -2797,10 +2789,14 @@
     <row r="64">
       <c r="A64" t="inlineStr">
         <is>
-          <t>Jesus Reyes</t>
-        </is>
-      </c>
-      <c r="B64" t="inlineStr"/>
+          <t>Sterling Clark</t>
+        </is>
+      </c>
+      <c r="B64" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
       <c r="C64" t="inlineStr">
         <is>
           <t>Yes</t>
@@ -2816,19 +2812,23 @@
           <t>Yes</t>
         </is>
       </c>
-      <c r="F64" t="inlineStr"/>
-      <c r="G64" t="inlineStr"/>
+      <c r="F64" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="G64" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
       <c r="H64" t="inlineStr">
         <is>
           <t>Yes</t>
         </is>
       </c>
       <c r="I64" t="inlineStr"/>
-      <c r="J64" t="inlineStr">
-        <is>
-          <t>Yes</t>
-        </is>
-      </c>
+      <c r="J64" t="inlineStr"/>
       <c r="K64" t="n">
         <v>4</v>
       </c>
@@ -2837,7 +2837,7 @@
     <row r="65">
       <c r="A65" t="inlineStr">
         <is>
-          <t>Sterling Clark</t>
+          <t>James May</t>
         </is>
       </c>
       <c r="B65" t="inlineStr">
@@ -2885,44 +2885,16 @@
     <row r="66">
       <c r="A66" t="inlineStr">
         <is>
-          <t>James May</t>
-        </is>
-      </c>
-      <c r="B66" t="inlineStr">
-        <is>
-          <t>Yes</t>
-        </is>
-      </c>
-      <c r="C66" t="inlineStr">
-        <is>
-          <t>Yes</t>
-        </is>
-      </c>
-      <c r="D66" t="inlineStr">
-        <is>
-          <t>Yes</t>
-        </is>
-      </c>
-      <c r="E66" t="inlineStr">
-        <is>
-          <t>Yes</t>
-        </is>
-      </c>
-      <c r="F66" t="inlineStr">
-        <is>
-          <t>Yes</t>
-        </is>
-      </c>
-      <c r="G66" t="inlineStr">
-        <is>
-          <t>Yes</t>
-        </is>
-      </c>
-      <c r="H66" t="inlineStr">
-        <is>
-          <t>Yes</t>
-        </is>
-      </c>
+          <t>James Dean</t>
+        </is>
+      </c>
+      <c r="B66" t="inlineStr"/>
+      <c r="C66" t="inlineStr"/>
+      <c r="D66" t="inlineStr"/>
+      <c r="E66" t="inlineStr"/>
+      <c r="F66" t="inlineStr"/>
+      <c r="G66" t="inlineStr"/>
+      <c r="H66" t="inlineStr"/>
       <c r="I66" t="inlineStr"/>
       <c r="J66" t="inlineStr"/>
       <c r="K66" t="n">
@@ -2933,7 +2905,7 @@
     <row r="67">
       <c r="A67" t="inlineStr">
         <is>
-          <t>James Dean</t>
+          <t>Cameron Manning</t>
         </is>
       </c>
       <c r="B67" t="inlineStr"/>
@@ -2953,15 +2925,23 @@
     <row r="68">
       <c r="A68" t="inlineStr">
         <is>
-          <t>Cameron Manning</t>
+          <t>Ericka McDaniel</t>
         </is>
       </c>
       <c r="B68" t="inlineStr"/>
       <c r="C68" t="inlineStr"/>
-      <c r="D68" t="inlineStr"/>
+      <c r="D68" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
       <c r="E68" t="inlineStr"/>
       <c r="F68" t="inlineStr"/>
-      <c r="G68" t="inlineStr"/>
+      <c r="G68" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
       <c r="H68" t="inlineStr"/>
       <c r="I68" t="inlineStr"/>
       <c r="J68" t="inlineStr"/>
@@ -2973,23 +2953,31 @@
     <row r="69">
       <c r="A69" t="inlineStr">
         <is>
-          <t>Ericka McDaniel</t>
-        </is>
-      </c>
-      <c r="B69" t="inlineStr"/>
+          <t>Mark Nicholas</t>
+        </is>
+      </c>
+      <c r="B69" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
       <c r="C69" t="inlineStr"/>
       <c r="D69" t="inlineStr">
         <is>
           <t>Yes</t>
         </is>
       </c>
-      <c r="E69" t="inlineStr"/>
-      <c r="F69" t="inlineStr"/>
-      <c r="G69" t="inlineStr">
-        <is>
-          <t>Yes</t>
-        </is>
-      </c>
+      <c r="E69" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="F69" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="G69" t="inlineStr"/>
       <c r="H69" t="inlineStr"/>
       <c r="I69" t="inlineStr"/>
       <c r="J69" t="inlineStr"/>
@@ -3001,7 +2989,7 @@
     <row r="70">
       <c r="A70" t="inlineStr">
         <is>
-          <t>Mark Nicholas</t>
+          <t>Connor Craven</t>
         </is>
       </c>
       <c r="B70" t="inlineStr">
@@ -3009,7 +2997,11 @@
           <t>Yes</t>
         </is>
       </c>
-      <c r="C70" t="inlineStr"/>
+      <c r="C70" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
       <c r="D70" t="inlineStr">
         <is>
           <t>Yes</t>
@@ -3025,8 +3017,16 @@
           <t>Yes</t>
         </is>
       </c>
-      <c r="G70" t="inlineStr"/>
-      <c r="H70" t="inlineStr"/>
+      <c r="G70" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="H70" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
       <c r="I70" t="inlineStr"/>
       <c r="J70" t="inlineStr"/>
       <c r="K70" t="n">
@@ -3037,7 +3037,7 @@
     <row r="71">
       <c r="A71" t="inlineStr">
         <is>
-          <t>Connor Craven</t>
+          <t>Mackay Callister</t>
         </is>
       </c>
       <c r="B71" t="inlineStr">
@@ -3085,7 +3085,7 @@
     <row r="72">
       <c r="A72" t="inlineStr">
         <is>
-          <t>Mackay Callister</t>
+          <t>Katrina Karlsson</t>
         </is>
       </c>
       <c r="B72" t="inlineStr">
@@ -3098,11 +3098,7 @@
           <t>Yes</t>
         </is>
       </c>
-      <c r="D72" t="inlineStr">
-        <is>
-          <t>Yes</t>
-        </is>
-      </c>
+      <c r="D72" t="inlineStr"/>
       <c r="E72" t="inlineStr">
         <is>
           <t>Yes</t>
@@ -3113,16 +3109,8 @@
           <t>Yes</t>
         </is>
       </c>
-      <c r="G72" t="inlineStr">
-        <is>
-          <t>Yes</t>
-        </is>
-      </c>
-      <c r="H72" t="inlineStr">
-        <is>
-          <t>Yes</t>
-        </is>
-      </c>
+      <c r="G72" t="inlineStr"/>
+      <c r="H72" t="inlineStr"/>
       <c r="I72" t="inlineStr"/>
       <c r="J72" t="inlineStr"/>
       <c r="K72" t="n">
@@ -3133,7 +3121,7 @@
     <row r="73">
       <c r="A73" t="inlineStr">
         <is>
-          <t>Katrina Karlsson</t>
+          <t>Edward Vidal</t>
         </is>
       </c>
       <c r="B73" t="inlineStr">
@@ -3147,17 +3135,17 @@
         </is>
       </c>
       <c r="D73" t="inlineStr"/>
-      <c r="E73" t="inlineStr">
-        <is>
-          <t>Yes</t>
-        </is>
-      </c>
+      <c r="E73" t="inlineStr"/>
       <c r="F73" t="inlineStr">
         <is>
           <t>Yes</t>
         </is>
       </c>
-      <c r="G73" t="inlineStr"/>
+      <c r="G73" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
       <c r="H73" t="inlineStr"/>
       <c r="I73" t="inlineStr"/>
       <c r="J73" t="inlineStr"/>
@@ -3169,7 +3157,7 @@
     <row r="74">
       <c r="A74" t="inlineStr">
         <is>
-          <t>Edward Vidal</t>
+          <t>Jacob Lampropoulos</t>
         </is>
       </c>
       <c r="B74" t="inlineStr">
@@ -3182,8 +3170,16 @@
           <t>Yes</t>
         </is>
       </c>
-      <c r="D74" t="inlineStr"/>
-      <c r="E74" t="inlineStr"/>
+      <c r="D74" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="E74" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
       <c r="F74" t="inlineStr">
         <is>
           <t>Yes</t>
@@ -3194,7 +3190,11 @@
           <t>Yes</t>
         </is>
       </c>
-      <c r="H74" t="inlineStr"/>
+      <c r="H74" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
       <c r="I74" t="inlineStr"/>
       <c r="J74" t="inlineStr"/>
       <c r="K74" t="n">
@@ -3205,7 +3205,7 @@
     <row r="75">
       <c r="A75" t="inlineStr">
         <is>
-          <t>Jacob Lampropoulos</t>
+          <t>Jake Barnes</t>
         </is>
       </c>
       <c r="B75" t="inlineStr">
@@ -3246,14 +3246,14 @@
       <c r="I75" t="inlineStr"/>
       <c r="J75" t="inlineStr"/>
       <c r="K75" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="L75" t="inlineStr"/>
     </row>
     <row r="76">
       <c r="A76" t="inlineStr">
         <is>
-          <t>Jake Barnes</t>
+          <t>Ian Bliss</t>
         </is>
       </c>
       <c r="B76" t="inlineStr">
@@ -3261,31 +3261,11 @@
           <t>Yes</t>
         </is>
       </c>
-      <c r="C76" t="inlineStr">
-        <is>
-          <t>Yes</t>
-        </is>
-      </c>
-      <c r="D76" t="inlineStr">
-        <is>
-          <t>Yes</t>
-        </is>
-      </c>
-      <c r="E76" t="inlineStr">
-        <is>
-          <t>Yes</t>
-        </is>
-      </c>
-      <c r="F76" t="inlineStr">
-        <is>
-          <t>Yes</t>
-        </is>
-      </c>
-      <c r="G76" t="inlineStr">
-        <is>
-          <t>Yes</t>
-        </is>
-      </c>
+      <c r="C76" t="inlineStr"/>
+      <c r="D76" t="inlineStr"/>
+      <c r="E76" t="inlineStr"/>
+      <c r="F76" t="inlineStr"/>
+      <c r="G76" t="inlineStr"/>
       <c r="H76" t="inlineStr">
         <is>
           <t>Yes</t>
@@ -3294,14 +3274,14 @@
       <c r="I76" t="inlineStr"/>
       <c r="J76" t="inlineStr"/>
       <c r="K76" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="L76" t="inlineStr"/>
     </row>
     <row r="77">
       <c r="A77" t="inlineStr">
         <is>
-          <t>Ian Bliss</t>
+          <t>Kameron Christofferson</t>
         </is>
       </c>
       <c r="B77" t="inlineStr">
@@ -3309,11 +3289,31 @@
           <t>Yes</t>
         </is>
       </c>
-      <c r="C77" t="inlineStr"/>
-      <c r="D77" t="inlineStr"/>
-      <c r="E77" t="inlineStr"/>
-      <c r="F77" t="inlineStr"/>
-      <c r="G77" t="inlineStr"/>
+      <c r="C77" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="D77" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="E77" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="F77" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="G77" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
       <c r="H77" t="inlineStr">
         <is>
           <t>Yes</t>
@@ -3329,7 +3329,7 @@
     <row r="78">
       <c r="A78" t="inlineStr">
         <is>
-          <t>Kameron Christofferson</t>
+          <t>Colten White</t>
         </is>
       </c>
       <c r="B78" t="inlineStr">
@@ -3377,87 +3377,71 @@
     <row r="79">
       <c r="A79" t="inlineStr">
         <is>
-          <t>Colten White</t>
-        </is>
-      </c>
-      <c r="B79" t="inlineStr">
-        <is>
-          <t>Yes</t>
-        </is>
-      </c>
+          <t>Rebecca Belt</t>
+        </is>
+      </c>
+      <c r="B79" t="inlineStr"/>
       <c r="C79" t="inlineStr">
         <is>
           <t>Yes</t>
         </is>
       </c>
-      <c r="D79" t="inlineStr">
-        <is>
-          <t>Yes</t>
-        </is>
-      </c>
-      <c r="E79" t="inlineStr">
-        <is>
-          <t>Yes</t>
-        </is>
-      </c>
+      <c r="D79" t="inlineStr"/>
+      <c r="E79" t="inlineStr"/>
       <c r="F79" t="inlineStr">
         <is>
           <t>Yes</t>
         </is>
       </c>
-      <c r="G79" t="inlineStr">
-        <is>
-          <t>Yes</t>
-        </is>
-      </c>
-      <c r="H79" t="inlineStr">
-        <is>
-          <t>Yes</t>
-        </is>
-      </c>
+      <c r="G79" t="inlineStr"/>
+      <c r="H79" t="inlineStr"/>
       <c r="I79" t="inlineStr"/>
-      <c r="J79" t="inlineStr"/>
+      <c r="J79" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
       <c r="K79" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="L79" t="inlineStr"/>
     </row>
     <row r="80">
       <c r="A80" t="inlineStr">
         <is>
-          <t>Rebecca Belt</t>
-        </is>
-      </c>
-      <c r="B80" t="inlineStr"/>
-      <c r="C80" t="inlineStr">
-        <is>
-          <t>Yes</t>
-        </is>
-      </c>
+          <t>Kristie Monroe</t>
+        </is>
+      </c>
+      <c r="B80" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="C80" t="inlineStr"/>
       <c r="D80" t="inlineStr"/>
       <c r="E80" t="inlineStr"/>
-      <c r="F80" t="inlineStr">
-        <is>
-          <t>Yes</t>
-        </is>
-      </c>
-      <c r="G80" t="inlineStr"/>
-      <c r="H80" t="inlineStr"/>
+      <c r="F80" t="inlineStr"/>
+      <c r="G80" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="H80" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
       <c r="I80" t="inlineStr"/>
-      <c r="J80" t="inlineStr">
-        <is>
-          <t>Yes</t>
-        </is>
-      </c>
+      <c r="J80" t="inlineStr"/>
       <c r="K80" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="L80" t="inlineStr"/>
     </row>
     <row r="81">
       <c r="A81" t="inlineStr">
         <is>
-          <t>Kristie Monroe</t>
+          <t>Chandler Vancott</t>
         </is>
       </c>
       <c r="B81" t="inlineStr">
@@ -3465,10 +3449,26 @@
           <t>Yes</t>
         </is>
       </c>
-      <c r="C81" t="inlineStr"/>
-      <c r="D81" t="inlineStr"/>
-      <c r="E81" t="inlineStr"/>
-      <c r="F81" t="inlineStr"/>
+      <c r="C81" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="D81" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="E81" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="F81" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
       <c r="G81" t="inlineStr">
         <is>
           <t>Yes</t>
@@ -3489,7 +3489,7 @@
     <row r="82">
       <c r="A82" t="inlineStr">
         <is>
-          <t>Chandler Vancott</t>
+          <t>Nathanael Anderson</t>
         </is>
       </c>
       <c r="B82" t="inlineStr">
@@ -3537,7 +3537,7 @@
     <row r="83">
       <c r="A83" t="inlineStr">
         <is>
-          <t>Nathanael Anderson</t>
+          <t>Sadie Dennis</t>
         </is>
       </c>
       <c r="B83" t="inlineStr">
@@ -3585,7 +3585,7 @@
     <row r="84">
       <c r="A84" t="inlineStr">
         <is>
-          <t>Sadie Dennis</t>
+          <t>Robert Luckau</t>
         </is>
       </c>
       <c r="B84" t="inlineStr">
@@ -3633,7 +3633,7 @@
     <row r="85">
       <c r="A85" t="inlineStr">
         <is>
-          <t>Robert Luckau</t>
+          <t>RJ Gomm</t>
         </is>
       </c>
       <c r="B85" t="inlineStr">
@@ -3674,14 +3674,14 @@
       <c r="I85" t="inlineStr"/>
       <c r="J85" t="inlineStr"/>
       <c r="K85" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="L85" t="inlineStr"/>
     </row>
     <row r="86">
       <c r="A86" t="inlineStr">
         <is>
-          <t>RJ Gomm</t>
+          <t>Aaron Henriksen</t>
         </is>
       </c>
       <c r="B86" t="inlineStr">
@@ -3720,9 +3720,13 @@
         </is>
       </c>
       <c r="I86" t="inlineStr"/>
-      <c r="J86" t="inlineStr"/>
+      <c r="J86" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
       <c r="K86" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="L86" t="inlineStr"/>
     </row>

</xml_diff>